<commit_message>
Direct generation of html
</commit_message>
<xml_diff>
--- a/tests/input/tech_radar.xlsx
+++ b/tests/input/tech_radar.xlsx
@@ -5,10 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Metadata" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Tech. List" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Sectors" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Zones" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="Trends" sheetId="5" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,9 +24,33 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="119">
-  <si>
-    <t xml:space="preserve">Date :</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="136">
+  <si>
+    <t xml:space="preserve">Title:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zalando Tech Radar </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Description:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zalando Tech Radar: a tool to visualize technology choices, inspire and support Engineering teams at Zalando to pick the best technologies for new projects </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Icon:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.zalando.de/favicon.ico </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repo url:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/zalando/tech-radar </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date:</t>
   </si>
   <si>
     <t xml:space="preserve">2025.05</t>
@@ -31,31 +59,34 @@
     <t xml:space="preserve">Active</t>
   </si>
   <si>
-    <t xml:space="preserve">Label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quadrant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ring</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
+    <t xml:space="preserve">Technology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tech. Sector</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monitoring Zone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trend</t>
   </si>
   <si>
     <t xml:space="preserve">Link</t>
   </si>
   <si>
+    <t xml:space="preserve">Comment</t>
+  </si>
+  <si>
     <t xml:space="preserve">X</t>
   </si>
   <si>
     <t xml:space="preserve">AWS Athena</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Datastores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Trial</t>
+    <t xml:space="preserve">Datastores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trial</t>
   </si>
   <si>
     <t xml:space="preserve">No change (●)</t>
@@ -64,13 +95,13 @@
     <t xml:space="preserve">AWS EMR</t>
   </si>
   <si>
-    <t xml:space="preserve">0. Adopt</t>
+    <t xml:space="preserve">Adopt</t>
   </si>
   <si>
     <t xml:space="preserve">AWS Glue</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Assess</t>
+    <t xml:space="preserve">Assess</t>
   </si>
   <si>
     <t xml:space="preserve">AWS Lake Formation</t>
@@ -112,7 +143,7 @@
     <t xml:space="preserve">AWS DocumentDB</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Data Management</t>
+    <t xml:space="preserve">Data Management</t>
   </si>
   <si>
     <t xml:space="preserve">AWS DynamoDB</t>
@@ -142,7 +173,7 @@
     <t xml:space="preserve">Apache Cassandra</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Hold</t>
+    <t xml:space="preserve">Hold</t>
   </si>
   <si>
     <t xml:space="preserve">https://engineering.zalando.com/tags/cassandra.html</t>
@@ -202,7 +233,7 @@
     <t xml:space="preserve">AWS CloudFormation</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Infrastructure</t>
+    <t xml:space="preserve">Infrastructure</t>
   </si>
   <si>
     <t xml:space="preserve">AWS CloudFront</t>
@@ -268,7 +299,7 @@
     <t xml:space="preserve">Clojure</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Languages</t>
+    <t xml:space="preserve">Languages</t>
   </si>
   <si>
     <t xml:space="preserve">https://engineering.zalando.com/tags/clojure.html</t>
@@ -377,6 +408,30 @@
   </si>
   <si>
     <t xml:space="preserve">https://engineering.zalando.com/tags/rabbitmq.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sector</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Color</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moved out (▼)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moved in (▲)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New (*)</t>
   </si>
 </sst>
 </file>
@@ -417,12 +472,36 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5BA300"/>
+        <bgColor rgb="FF339966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF009EB0"/>
+        <bgColor rgb="FF008080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC7BA00"/>
+        <bgColor rgb="FFFFCC00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE09B96"/>
+        <bgColor rgb="FFFF8080"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -466,7 +545,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -475,8 +554,44 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -488,7 +603,75 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF5BA300"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF009EB0"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFE09B96"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FFC7BA00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Trends" displayName="Trends" ref="A2:A5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <tableColumns count="1">
+    <tableColumn id="1" name="Moved out (▼)"/>
+  </tableColumns>
+</table>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -496,15 +679,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F79"/>
-  <sheetFormatPr defaultColWidth="8.61328125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="27.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="46.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="71.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -514,1418 +693,1499 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G1048576"/>
+  <sheetFormatPr defaultColWidth="8.65234375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="46.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10.2"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>8</v>
+      <c r="A3" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>8</v>
+      <c r="A4" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>8</v>
+      <c r="A5" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>8</v>
+      <c r="A6" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>8</v>
+      <c r="A7" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>8</v>
+      <c r="A8" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B8" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="0" t="s">
-        <v>10</v>
-      </c>
       <c r="D8" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>8</v>
+      <c r="A9" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B9" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>14</v>
-      </c>
       <c r="E9" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="F9" s="0" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>8</v>
+      <c r="A10" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="0" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>8</v>
+      <c r="A11" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>8</v>
+      <c r="A12" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="F12" s="0" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>8</v>
+      <c r="A13" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B13" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>14</v>
-      </c>
       <c r="E13" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="0" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>8</v>
+      <c r="A14" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>8</v>
+      <c r="A15" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>8</v>
+      <c r="A16" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
-        <v>8</v>
+      <c r="A17" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
-        <v>8</v>
+      <c r="A18" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="F18" s="0" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
-        <v>8</v>
+      <c r="A19" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F19" s="0" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
-        <v>8</v>
+      <c r="A20" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
-        <v>8</v>
+      <c r="A21" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
-        <v>8</v>
+      <c r="A22" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
-        <v>8</v>
+      <c r="A23" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="F23" s="0" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
-        <v>8</v>
+      <c r="A24" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F24" s="0" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
-        <v>8</v>
+      <c r="A25" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
-        <v>8</v>
+      <c r="A26" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B26" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E26" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26" s="0" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="D27" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="E27" s="0" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="D28" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="E28" s="0" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B29" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="E29" s="0" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B30" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="D30" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="E30" s="0" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B31" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="D31" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="E31" s="0" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B32" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="D32" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="E32" s="0" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B33" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="C33" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="D33" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="E33" s="0" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B34" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="C34" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="D34" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E34" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="F34" s="0" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B35" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="C35" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="D35" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="E35" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="C26" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D26" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B27" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D27" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="E27" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F27" s="0" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B28" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="C28" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D28" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="E28" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B29" s="0" t="s">
-        <v>47</v>
-      </c>
-      <c r="C29" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D29" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="E29" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B30" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="C30" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D30" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="E30" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B31" s="0" t="s">
+    </row>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B36" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="D36" s="0" t="s">
         <v>49</v>
       </c>
-      <c r="C31" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D31" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="E31" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B32" s="0" t="s">
-        <v>50</v>
-      </c>
-      <c r="C32" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D32" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="E32" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B33" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="C33" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D33" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="E33" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B34" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="C34" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D34" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="E34" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B35" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="C35" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D35" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="E35" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F35" s="0" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B36" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="C36" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D36" s="0" t="s">
-        <v>40</v>
-      </c>
       <c r="E36" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F36" s="0" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
-        <v>8</v>
+      <c r="A37" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="F37" s="0" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
-        <v>8</v>
+      <c r="A38" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F38" s="0" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
-        <v>8</v>
+      <c r="A39" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
-        <v>8</v>
+      <c r="A40" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
-        <v>8</v>
+      <c r="A41" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
-        <v>8</v>
+      <c r="A42" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0" t="s">
-        <v>8</v>
+      <c r="A43" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="E43" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
-        <v>8</v>
+      <c r="A44" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E44" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
-        <v>8</v>
+      <c r="A45" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="E45" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0" t="s">
-        <v>8</v>
+      <c r="A46" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0" t="s">
-        <v>8</v>
+      <c r="A47" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="0" t="s">
-        <v>8</v>
+      <c r="A48" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C48" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="F48" s="0" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="0" t="s">
-        <v>8</v>
+      <c r="A49" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B49" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="C49" s="0" t="s">
         <v>69</v>
       </c>
-      <c r="C49" s="0" t="s">
-        <v>60</v>
-      </c>
       <c r="D49" s="0" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F49" s="0" t="s">
-        <v>70</v>
+        <v>21</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="0" t="s">
-        <v>8</v>
+      <c r="A50" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C50" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D50" s="0" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E50" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="0" t="s">
-        <v>8</v>
+      <c r="A51" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="E51" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="F51" s="0" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="0" t="s">
-        <v>8</v>
+      <c r="A52" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F52" s="0" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="0" t="s">
-        <v>8</v>
+      <c r="A53" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D53" s="0" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E53" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="0" t="s">
-        <v>8</v>
+      <c r="A54" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E54" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="0" t="s">
-        <v>8</v>
+      <c r="A55" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="0" t="s">
-        <v>8</v>
+      <c r="A56" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E56" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="0" t="s">
-        <v>8</v>
+      <c r="A57" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E57" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="0" t="s">
-        <v>8</v>
+      <c r="A58" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="E58" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="F58" s="0" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="0" t="s">
-        <v>8</v>
+      <c r="A59" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F59" s="0" t="s">
-        <v>83</v>
+        <v>21</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="0" t="s">
-        <v>8</v>
+      <c r="A60" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="F60" s="0" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="0" t="s">
-        <v>8</v>
+      <c r="A61" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E61" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F61" s="0" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="0" t="s">
-        <v>8</v>
+      <c r="A62" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="E62" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F62" s="0" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="0" t="s">
-        <v>8</v>
+      <c r="A63" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="E63" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F63" s="0" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="0" t="s">
-        <v>8</v>
+      <c r="A64" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B64" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="C64" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="C64" s="0" t="s">
-        <v>82</v>
-      </c>
       <c r="D64" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E64" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F64" s="0" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0" t="s">
-        <v>8</v>
+      <c r="A65" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E65" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F65" s="0" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="0" t="s">
-        <v>8</v>
+      <c r="A66" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E66" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F66" s="0" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="0" t="s">
-        <v>8</v>
+      <c r="A67" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E67" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F67" s="0" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0" t="s">
-        <v>8</v>
+      <c r="A68" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D68" s="0" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E68" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F68" s="0" t="s">
-        <v>100</v>
+        <v>21</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0" t="s">
-        <v>8</v>
+      <c r="A69" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B69" s="0" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="C69" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D69" s="0" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="E69" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="F69" s="0" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="0" t="s">
-        <v>8</v>
+      <c r="A70" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B70" s="0" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="C70" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D70" s="0" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="E70" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F70" s="0" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="0" t="s">
-        <v>8</v>
+      <c r="A71" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B71" s="0" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="C71" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D71" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E71" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F71" s="0" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="0" t="s">
-        <v>8</v>
+      <c r="A72" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B72" s="0" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="C72" s="0" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="D72" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E72" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F72" s="0" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="0" t="s">
-        <v>8</v>
+      <c r="A73" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B73" s="0" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="C73" s="0" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D73" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E73" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F73" s="0" t="s">
-        <v>109</v>
+        <v>21</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="0" t="s">
-        <v>8</v>
+      <c r="A74" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B74" s="0" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="C74" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D74" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E74" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="0" t="s">
-        <v>8</v>
+      <c r="A75" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D75" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E75" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="0" t="s">
-        <v>8</v>
+      <c r="A76" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="C76" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D76" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E76" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="F76" s="0" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="0" t="s">
-        <v>8</v>
+      <c r="A77" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B77" s="0" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="C77" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D77" s="0" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E77" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F77" s="0" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="0" t="s">
-        <v>8</v>
+      <c r="A78" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="B78" s="0" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="C78" s="0" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D78" s="0" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E78" s="0" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F78" s="0" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B79" s="0" t="s">
-        <v>117</v>
-      </c>
-      <c r="C79" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D79" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="E79" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F79" s="0" t="s">
-        <v>118</v>
-      </c>
-    </row>
+        <v>127</v>
+      </c>
+    </row>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -1935,4 +2195,186 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.07"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="5.36"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="6"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="7"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="8"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="9"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.15"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>135</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+  <tableParts>
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>